<commit_message>
Update TEST Assignment 1 - Test cases.xlsx
</commit_message>
<xml_diff>
--- a/IT23321618/TEST Assignment 1 - Test cases.xlsx
+++ b/IT23321618/TEST Assignment 1 - Test cases.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pramo\OneDrive\Desktop\IT23321618\IT23321618\IT23321618\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\testing\IT23321618\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{348457C0-6629-4A6D-A8F1-7C1616AADAC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5EB761B-F899-4ABB-8EFB-EC09CFFE5C38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="12210" windowHeight="12885" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name=" Test cases" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="282">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -638,6 +638,234 @@
   </si>
   <si>
     <t>හවස 3.30 ප.ව එන්න</t>
+  </si>
+  <si>
+    <t>Singlish input types covered</t>
+  </si>
+  <si>
+    <t>Evidence or rationale</t>
+  </si>
+  <si>
+    <t>English insertions</t>
+  </si>
+  <si>
+    <t>Word 'practical' not transliterated</t>
+  </si>
+  <si>
+    <t>Abbreviations</t>
+  </si>
+  <si>
+    <t>PDF abbreviation preserved incorrectly</t>
+  </si>
+  <si>
+    <t>Negation forms</t>
+  </si>
+  <si>
+    <t>Negation 'ne' — 'hari ne' pattern</t>
+  </si>
+  <si>
+    <t>Romanization</t>
+  </si>
+  <si>
+    <t>mn' variation for 'mang'</t>
+  </si>
+  <si>
+    <t>API abbreviation</t>
+  </si>
+  <si>
+    <t>Capitalisation variation</t>
+  </si>
+  <si>
+    <t>Mid-sentence capital causes incorrect output</t>
+  </si>
+  <si>
+    <t>Clipped forms</t>
+  </si>
+  <si>
+    <t>bona oni' short form for 'bonna one'</t>
+  </si>
+  <si>
+    <t>Semantic mismatch</t>
+  </si>
+  <si>
+    <t>Unrelated output returned for input</t>
+  </si>
+  <si>
+    <t>Word 'train' not transliterated</t>
+  </si>
+  <si>
+    <t>Slang dates</t>
+  </si>
+  <si>
+    <t>2moro' informal for 'tomorrow'</t>
+  </si>
+  <si>
+    <t>Numbers</t>
+  </si>
+  <si>
+    <t>Large number word 'harasiya panaha' not fully converted</t>
+  </si>
+  <si>
+    <t>Word boundary</t>
+  </si>
+  <si>
+    <t>Ambiguous compound 'matahari' (mata + hari)</t>
+  </si>
+  <si>
+    <t>Repeated characters</t>
+  </si>
+  <si>
+    <t>Extended vowel 'yananoooo' in input</t>
+  </si>
+  <si>
+    <t>Missing space: 'eyagiya' (eya + giya)</t>
+  </si>
+  <si>
+    <t>Pronoun variation</t>
+  </si>
+  <si>
+    <t>Demonstrative pronoun 'eka' vs 'eka'</t>
+  </si>
+  <si>
+    <t>Word 'phone' not transliterated to 'fone'</t>
+  </si>
+  <si>
+    <t>Word 'school' not converted to Sinhala</t>
+  </si>
+  <si>
+    <t>Word 'run' not transliterated</t>
+  </si>
+  <si>
+    <t>Question forms</t>
+  </si>
+  <si>
+    <t>yawanawada' question marker</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>5.30 PM' time not converted to 'ප.ව'</t>
+  </si>
+  <si>
+    <t>kohomada' interrogative form</t>
+  </si>
+  <si>
+    <t>harii ne' — negation with emphasis</t>
+  </si>
+  <si>
+    <t>Ordinal '8th' not converted correctly</t>
+  </si>
+  <si>
+    <t>Informal spelling 'uba', 'baqq'</t>
+  </si>
+  <si>
+    <t>Spelling variant 'samanera hima'</t>
+  </si>
+  <si>
+    <t>Online identifiers</t>
+  </si>
+  <si>
+    <t>Email address in input</t>
+  </si>
+  <si>
+    <t>Password with alphanumeric string</t>
+  </si>
+  <si>
+    <t>Place names</t>
+  </si>
+  <si>
+    <t>Place name 'maathara' (Matara)</t>
+  </si>
+  <si>
+    <t>Formal/Religious language</t>
+  </si>
+  <si>
+    <t>Religious term 'suraameerayen'</t>
+  </si>
+  <si>
+    <t>Emojis</t>
+  </si>
+  <si>
+    <t>Emoji 😍 in input</t>
+  </si>
+  <si>
+    <t>Measurements</t>
+  </si>
+  <si>
+    <t>50 KG' not converted to Sinhala unit</t>
+  </si>
+  <si>
+    <t>English phrases</t>
+  </si>
+  <si>
+    <t>best wishes' phrase in input</t>
+  </si>
+  <si>
+    <t>eyi' variation + English insertion 'bro'</t>
+  </si>
+  <si>
+    <t>Missing space: 'malliheta' (malli + heta)</t>
+  </si>
+  <si>
+    <t>Emoji 🤔 swapped to 😅 in output</t>
+  </si>
+  <si>
+    <t>NIC abbreviation</t>
+  </si>
+  <si>
+    <t>Slang</t>
+  </si>
+  <si>
+    <t>ela ela' colloquial expression + emoji 👍</t>
+  </si>
+  <si>
+    <t>Email address incorrectly transliterated</t>
+  </si>
+  <si>
+    <t>URL not preserved in output</t>
+  </si>
+  <si>
+    <t>2day' informal for 'today'</t>
+  </si>
+  <si>
+    <t>Punctuation</t>
+  </si>
+  <si>
+    <t>Double '??' + question form 'harida'</t>
+  </si>
+  <si>
+    <t>3.30 pm' time expression not converted</t>
+  </si>
+  <si>
+    <t>Currency</t>
+  </si>
+  <si>
+    <t>'USD 100' currency not converted to Sinhala</t>
+  </si>
+  <si>
+    <t>Ordinal '5th' not converted correctly</t>
+  </si>
+  <si>
+    <t>scene ekak' — colloquial English insertion</t>
+  </si>
+  <si>
+    <t>NIC number + greeting + email in input</t>
+  </si>
+  <si>
+    <t>Dates</t>
+  </si>
+  <si>
+    <t>Month name 'November 15' not converted</t>
+  </si>
+  <si>
+    <t>oone' spelling variant of 'one'</t>
+  </si>
+  <si>
+    <t>RS 200' currency not converted to Sinhala</t>
+  </si>
+  <si>
+    <t>All words concatenated without spaces</t>
   </si>
 </sst>
 </file>
@@ -757,7 +985,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -766,6 +993,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1047,7 +1277,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr defaultRowHeight="49.9" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.85546875" customWidth="1"/>
@@ -1055,11 +1285,11 @@
     <col min="4" max="4" width="25.28515625" customWidth="1"/>
     <col min="5" max="5" width="28.42578125" customWidth="1"/>
     <col min="7" max="7" width="31.5703125" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="8" max="8" width="40.140625" customWidth="1"/>
     <col min="9" max="10" width="12.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1078,16 +1308,21 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6"/>
-    </row>
-    <row r="2" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+      <c r="G1" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="7" t="s">
         <v>8</v>
       </c>
       <c r="D2" s="5" t="s">
@@ -1099,15 +1334,21 @@
       <c r="F2" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="G2" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
         <v>11</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="7" t="s">
         <v>12</v>
       </c>
       <c r="D3" s="5" t="s">
@@ -1119,15 +1360,21 @@
       <c r="F3" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+      <c r="G3" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>16</v>
       </c>
       <c r="D4" s="5" t="s">
@@ -1139,15 +1386,21 @@
       <c r="F4" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="G4" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
         <v>19</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="7" t="s">
         <v>20</v>
       </c>
       <c r="D5" s="5" t="s">
@@ -1159,15 +1412,21 @@
       <c r="F5" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="G5" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
         <v>23</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="7" t="s">
         <v>24</v>
       </c>
       <c r="D6" s="3" t="s">
@@ -1179,15 +1438,21 @@
       <c r="F6" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+      <c r="G6" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
         <v>27</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="7" t="s">
         <v>28</v>
       </c>
       <c r="D7" s="3" t="s">
@@ -1199,15 +1464,21 @@
       <c r="F7" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+      <c r="G7" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
         <v>31</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="7" t="s">
         <v>32</v>
       </c>
       <c r="D8" s="3" t="s">
@@ -1219,15 +1490,21 @@
       <c r="F8" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
+      <c r="G8" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
         <v>34</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="7" t="s">
         <v>35</v>
       </c>
       <c r="D9" s="3" t="s">
@@ -1239,15 +1516,21 @@
       <c r="F9" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
+      <c r="G9" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
         <v>38</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="7" t="s">
         <v>39</v>
       </c>
       <c r="D10" s="3" t="s">
@@ -1259,15 +1542,21 @@
       <c r="F10" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
+      <c r="G10" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
         <v>41</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="7" t="s">
         <v>43</v>
       </c>
       <c r="D11" s="3" t="s">
@@ -1279,15 +1568,21 @@
       <c r="F11" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
+      <c r="G11" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
         <v>45</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="7" t="s">
         <v>46</v>
       </c>
       <c r="D12" s="3" t="s">
@@ -1299,15 +1594,21 @@
       <c r="F12" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
+      <c r="G12" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
         <v>48</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="7" t="s">
         <v>49</v>
       </c>
       <c r="D13" s="3" t="s">
@@ -1319,15 +1620,21 @@
       <c r="F13" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
+      <c r="G13" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
         <v>51</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="7" t="s">
         <v>52</v>
       </c>
       <c r="D14" s="3" t="s">
@@ -1339,15 +1646,21 @@
       <c r="F14" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
+      <c r="G14" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
         <v>54</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="7" t="s">
         <v>55</v>
       </c>
       <c r="D15" s="3" t="s">
@@ -1359,15 +1672,21 @@
       <c r="F15" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
+      <c r="G15" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
         <v>57</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="7" t="s">
         <v>58</v>
       </c>
       <c r="D16" s="3" t="s">
@@ -1379,15 +1698,21 @@
       <c r="F16" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
+      <c r="G16" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
         <v>60</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="7" t="s">
         <v>61</v>
       </c>
       <c r="D17" s="3" t="s">
@@ -1399,15 +1724,21 @@
       <c r="F17" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
+      <c r="G17" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
         <v>64</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="7" t="s">
         <v>65</v>
       </c>
       <c r="D18" s="3" t="s">
@@ -1419,15 +1750,21 @@
       <c r="F18" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
+      <c r="G18" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
         <v>67</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="7" t="s">
         <v>68</v>
       </c>
       <c r="D19" s="3" t="s">
@@ -1439,15 +1776,21 @@
       <c r="F19" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="7" t="s">
+      <c r="G19" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
         <v>71</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="7" t="s">
         <v>72</v>
       </c>
       <c r="D20" s="3" t="s">
@@ -1459,15 +1802,21 @@
       <c r="F20" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="7" t="s">
+      <c r="G20" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="H20" s="10" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
         <v>74</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="C21" s="7" t="s">
         <v>75</v>
       </c>
       <c r="D21" s="3" t="s">
@@ -1479,15 +1828,21 @@
       <c r="F21" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
+      <c r="G21" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="H21" s="10" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
         <v>77</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="7" t="s">
         <v>78</v>
       </c>
       <c r="D22" s="3" t="s">
@@ -1499,15 +1854,21 @@
       <c r="F22" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="7" t="s">
+      <c r="G22" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="H22" s="10" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
         <v>80</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="7" t="s">
         <v>176</v>
       </c>
       <c r="D23" s="3" t="s">
@@ -1519,15 +1880,21 @@
       <c r="F23" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="7" t="s">
+      <c r="G23" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="H23" s="10" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="6" t="s">
         <v>81</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="7" t="s">
         <v>82</v>
       </c>
       <c r="D24" s="3" t="s">
@@ -1539,15 +1906,21 @@
       <c r="F24" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="7" t="s">
+      <c r="G24" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="6" t="s">
         <v>85</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="7" t="s">
         <v>86</v>
       </c>
       <c r="D25" s="3" t="s">
@@ -1559,15 +1932,21 @@
       <c r="F25" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="7" t="s">
+      <c r="G25" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="6" t="s">
         <v>88</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D26" s="3" t="s">
@@ -1579,15 +1958,21 @@
       <c r="F26" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="7" t="s">
+      <c r="G26" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="6" t="s">
         <v>92</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="7" t="s">
         <v>93</v>
       </c>
       <c r="D27" s="3" t="s">
@@ -1599,15 +1984,21 @@
       <c r="F27" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="7" t="s">
+      <c r="G27" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="6" t="s">
         <v>96</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C28" s="8" t="s">
+      <c r="C28" s="7" t="s">
         <v>97</v>
       </c>
       <c r="D28" s="3" t="s">
@@ -1619,15 +2010,21 @@
       <c r="F28" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="7" t="s">
+      <c r="G28" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="6" t="s">
         <v>100</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C29" s="8" t="s">
+      <c r="C29" s="7" t="s">
         <v>101</v>
       </c>
       <c r="D29" s="3" t="s">
@@ -1639,18 +2036,24 @@
       <c r="F29" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="7" t="s">
+      <c r="G29" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="6" t="s">
         <v>104</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C30" s="8" t="s">
+      <c r="C30" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="D30" s="10" t="s">
+      <c r="D30" s="9" t="s">
         <v>106</v>
       </c>
       <c r="E30" s="2" t="s">
@@ -1659,15 +2062,21 @@
       <c r="F30" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="7" t="s">
+      <c r="G30" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
         <v>107</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C31" s="8" t="s">
+      <c r="C31" s="7" t="s">
         <v>108</v>
       </c>
       <c r="D31" s="3" t="s">
@@ -1679,15 +2088,21 @@
       <c r="F31" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="7" t="s">
+      <c r="G31" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="H31" s="4" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="6" t="s">
         <v>110</v>
       </c>
       <c r="B32" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C32" s="8" t="s">
+      <c r="C32" s="7" t="s">
         <v>111</v>
       </c>
       <c r="D32" s="3" t="s">
@@ -1699,15 +2114,21 @@
       <c r="F32" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="7" t="s">
+      <c r="G32" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="H32" s="10" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="6" t="s">
         <v>113</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C33" s="8" t="s">
+      <c r="C33" s="7" t="s">
         <v>114</v>
       </c>
       <c r="D33" s="3" t="s">
@@ -1719,15 +2140,21 @@
       <c r="F33" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="7" t="s">
+      <c r="G33" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="H33" s="10" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="6" t="s">
         <v>117</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C34" s="8" t="s">
+      <c r="C34" s="7" t="s">
         <v>118</v>
       </c>
       <c r="D34" s="3" t="s">
@@ -1739,15 +2166,21 @@
       <c r="F34" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="7" t="s">
+      <c r="G34" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="H34" s="10" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="6" t="s">
         <v>121</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C35" s="8" t="s">
+      <c r="C35" s="7" t="s">
         <v>122</v>
       </c>
       <c r="D35" s="3" t="s">
@@ -1759,15 +2192,21 @@
       <c r="F35" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="7" t="s">
+      <c r="G35" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="6" t="s">
         <v>125</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C36" s="8" t="s">
+      <c r="C36" s="7" t="s">
         <v>126</v>
       </c>
       <c r="D36" s="3" t="s">
@@ -1779,15 +2218,21 @@
       <c r="F36" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="7" t="s">
+      <c r="G36" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="H36" s="4" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="6" t="s">
         <v>129</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C37" s="8" t="s">
+      <c r="C37" s="7" t="s">
         <v>130</v>
       </c>
       <c r="D37" s="3" t="s">
@@ -1799,15 +2244,21 @@
       <c r="F37" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="7" t="s">
+      <c r="G37" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="H37" s="4" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="6" t="s">
         <v>133</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C38" s="8" t="s">
+      <c r="C38" s="7" t="s">
         <v>134</v>
       </c>
       <c r="D38" s="3" t="s">
@@ -1819,35 +2270,47 @@
       <c r="F38" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="7" t="s">
+      <c r="G38" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="H38" s="10" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="6" t="s">
         <v>137</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C39" s="9" t="s">
+      <c r="C39" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="D39" s="9" t="s">
+      <c r="D39" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="E39" s="9" t="s">
+      <c r="E39" s="8" t="s">
         <v>197</v>
       </c>
       <c r="F39" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="7" t="s">
+      <c r="G39" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="H39" s="4" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="6" t="s">
         <v>140</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C40" s="8" t="s">
+      <c r="C40" s="7" t="s">
         <v>141</v>
       </c>
       <c r="D40" s="3" t="s">
@@ -1859,15 +2322,21 @@
       <c r="F40" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="7" t="s">
+      <c r="G40" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="H40" s="4" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="6" t="s">
         <v>142</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C41" s="8" t="s">
+      <c r="C41" s="7" t="s">
         <v>143</v>
       </c>
       <c r="D41" s="3" t="s">
@@ -1879,15 +2348,21 @@
       <c r="F41" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="7" t="s">
+      <c r="G41" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="H41" s="10" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="6" t="s">
         <v>145</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C42" s="8" t="s">
+      <c r="C42" s="7" t="s">
         <v>146</v>
       </c>
       <c r="D42" s="3" t="s">
@@ -1899,15 +2374,21 @@
       <c r="F42" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="7" t="s">
+      <c r="G42" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="H42" s="4" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="6" t="s">
         <v>148</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C43" s="8" t="s">
+      <c r="C43" s="7" t="s">
         <v>203</v>
       </c>
       <c r="D43" s="3" t="s">
@@ -1919,15 +2400,21 @@
       <c r="F43" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="7" t="s">
+      <c r="G43" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="H43" s="10" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="6" t="s">
         <v>149</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C44" s="8" t="s">
+      <c r="C44" s="7" t="s">
         <v>150</v>
       </c>
       <c r="D44" s="3" t="s">
@@ -1939,15 +2426,21 @@
       <c r="F44" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="7" t="s">
+      <c r="G44" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="H44" s="4" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="6" t="s">
         <v>152</v>
       </c>
       <c r="B45" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C45" s="8" t="s">
+      <c r="C45" s="7" t="s">
         <v>153</v>
       </c>
       <c r="D45" s="3" t="s">
@@ -1959,15 +2452,21 @@
       <c r="F45" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="7" t="s">
+      <c r="G45" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="6" t="s">
         <v>155</v>
       </c>
       <c r="B46" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C46" s="8" t="s">
+      <c r="C46" s="7" t="s">
         <v>156</v>
       </c>
       <c r="D46" s="3" t="s">
@@ -1979,15 +2478,21 @@
       <c r="F46" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="7" t="s">
+      <c r="G46" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="H46" s="10" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="6" t="s">
         <v>159</v>
       </c>
       <c r="B47" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C47" s="8" t="s">
+      <c r="C47" s="7" t="s">
         <v>160</v>
       </c>
       <c r="D47" s="3" t="s">
@@ -1999,15 +2504,21 @@
       <c r="F47" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="7" t="s">
+      <c r="G47" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="H47" s="4" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="6" t="s">
         <v>163</v>
       </c>
       <c r="B48" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C48" s="8" t="s">
+      <c r="C48" s="7" t="s">
         <v>164</v>
       </c>
       <c r="D48" s="3" t="s">
@@ -2019,15 +2530,21 @@
       <c r="F48" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="7" t="s">
+      <c r="G48" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="H48" s="4" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="6" t="s">
         <v>166</v>
       </c>
       <c r="B49" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C49" s="8" t="s">
+      <c r="C49" s="7" t="s">
         <v>167</v>
       </c>
       <c r="D49" s="3" t="s">
@@ -2039,15 +2556,21 @@
       <c r="F49" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="7" t="s">
+      <c r="G49" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="H49" s="10" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="6" t="s">
         <v>169</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C50" s="8" t="s">
+      <c r="C50" s="7" t="s">
         <v>170</v>
       </c>
       <c r="D50" s="3" t="s">
@@ -2059,15 +2582,21 @@
       <c r="F50" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="7" t="s">
+      <c r="G50" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="H50" s="10" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="6" t="s">
         <v>173</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C51" s="8" t="s">
+      <c r="C51" s="7" t="s">
         <v>174</v>
       </c>
       <c r="D51" s="3" t="s">
@@ -2078,6 +2607,12 @@
       </c>
       <c r="F51" s="4" t="s">
         <v>10</v>
+      </c>
+      <c r="G51" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="H51" s="4" t="s">
+        <v>281</v>
       </c>
     </row>
   </sheetData>

</xml_diff>